<commit_message>
EPBDS-9967 Read a whole number with leading zeros as decimal, so 08, 09, 008 and 009 compile
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
@@ -583,14 +583,14 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Formulas accept Java-like literals, written in digits only. A whole number is an Integer, "L" makes it a Long, "0x" starts a hexadecimal number, a leading zero an octal one, a dot or an exponent makes a Double, "f" a Float, and "%" divides by 100 exactly, with any number of decimals.</t>
+          <t>Formulas accept Java-like literals, written in digits only. A whole number is an Integer, "L" makes it a Long, "0x" starts a hexadecimal number, leading zeros keep a number decimal, a dot or an exponent makes a Double, "f" a Float, and "%" divides by 100 exactly, with any number of decimals.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. "$" starts a reference to a spreadsheet step, so it cannot start a number, and K, M, B are not multipliers. Range cells accept these forms, see the ValuesAndRanges workbook. A leading zero makes 08 and 09 invalid: write Date(2021, 4, 8), not Date(2021, 04, 08).</t>
+          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. "$" starts a reference to a spreadsheet step, so it cannot start a number, and K, M, B are not multipliers. Range cells accept these forms, see the ValuesAndRanges workbook. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
         </is>
       </c>
     </row>
@@ -653,7 +653,7 @@
     <row r="13">
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Octal</t>
+          <t>LeadingZeros</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>_res_.$Octal</t>
+          <t>_res_.$LeadingZeros</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
@@ -1026,7 +1026,7 @@
         <v>255</v>
       </c>
       <c r="E31" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F31" s="10" t="n">
         <v>1.5</v>

</xml_diff>

<commit_message>
Fix lexical error on Korean names caused by fixed Unicode ranges of identifiers
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
@@ -12,9 +12,40 @@
     <sheet name="Casts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Calls" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>Method Double 면간거리(Double 폭, Double 간격)</t>
+  </si>
+  <si>
+    <t>return 폭 + 간격;</t>
+  </si>
+  <si>
+    <t>Test 면간거리 면간거리Test</t>
+  </si>
+  <si>
+    <t>폭</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t>간격</t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
+    <t>_res_</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -553,24 +584,24 @@
   <dimension ref="B2:R49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="24.7" customWidth="1" min="2" max="2"/>
-    <col width="27.9" customWidth="1" min="3" max="3"/>
-    <col width="20.9" customWidth="1" min="4" max="4"/>
-    <col width="21.9" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="17.8" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="20.9" customWidth="1" min="9" max="9"/>
-    <col width="16.7" customWidth="1" min="10" max="10"/>
-    <col width="16.7" customWidth="1" min="11" max="11"/>
-    <col width="25.1" customWidth="1" min="12" max="12"/>
-    <col width="25.1" customWidth="1" min="13" max="13"/>
-    <col width="27.2" customWidth="1" min="14" max="14"/>
-    <col width="30.4" customWidth="1" min="15" max="15"/>
-    <col width="21.9" customWidth="1" min="16" max="16"/>
-    <col width="21.9" customWidth="1" min="17" max="17"/>
-    <col width="24.1" customWidth="1" min="18" max="18"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="24.7"/>
+    <col min="3" max="3" customWidth="true" width="27.9"/>
+    <col min="4" max="4" customWidth="true" width="20.9"/>
+    <col min="5" max="5" customWidth="true" width="21.9"/>
+    <col min="6" max="6" customWidth="true" width="23.0"/>
+    <col min="7" max="7" customWidth="true" width="17.8"/>
+    <col min="8" max="8" customWidth="true" width="23.0"/>
+    <col min="9" max="9" customWidth="true" width="20.9"/>
+    <col min="10" max="10" customWidth="true" width="16.7"/>
+    <col min="11" max="11" customWidth="true" width="16.7"/>
+    <col min="12" max="12" customWidth="true" width="25.1"/>
+    <col min="13" max="13" customWidth="true" width="25.1"/>
+    <col min="14" max="14" customWidth="true" width="27.2"/>
+    <col min="15" max="15" customWidth="true" width="30.4"/>
+    <col min="16" max="16" customWidth="true" width="21.9"/>
+    <col min="17" max="17" customWidth="true" width="21.9"/>
+    <col min="18" max="18" customWidth="true" width="24.1"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1346,15 +1377,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I16"/>
+  <dimension ref="B2:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="16.8" customWidth="1" min="2" max="2"/>
-    <col width="72.2" customWidth="1" min="3" max="3"/>
-    <col width="14.6" customWidth="1" min="4" max="4"/>
-    <col width="21.9" customWidth="1" min="5" max="5"/>
-    <col width="21.9" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="16.8"/>
+    <col min="3" max="3" customWidth="true" width="72.2"/>
+    <col min="4" max="4" customWidth="true" width="14.6"/>
+    <col min="5" max="5" customWidth="true" width="21.9"/>
+    <col min="6" max="6" customWidth="true" width="21.9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1546,15 +1577,15 @@
   <dimension ref="B2:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="42.7" customWidth="1" min="2" max="2"/>
-    <col width="50.3" customWidth="1" min="3" max="3"/>
-    <col width="15.7" customWidth="1" min="4" max="4"/>
-    <col width="21.9" customWidth="1" min="5" max="5"/>
-    <col width="25.1" customWidth="1" min="6" max="6"/>
-    <col width="14.6" customWidth="1" min="7" max="7"/>
-    <col width="15.7" customWidth="1" min="8" max="8"/>
-    <col width="19.9" customWidth="1" min="9" max="9"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="42.7"/>
+    <col min="3" max="3" customWidth="true" width="50.3"/>
+    <col min="4" max="4" customWidth="true" width="15.7"/>
+    <col min="5" max="5" customWidth="true" width="21.9"/>
+    <col min="6" max="6" customWidth="true" width="25.1"/>
+    <col min="7" max="7" customWidth="true" width="14.6"/>
+    <col min="8" max="8" customWidth="true" width="15.7"/>
+    <col min="9" max="9" customWidth="true" width="19.9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1909,15 +1940,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I23"/>
+  <dimension ref="B2:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="68" customWidth="1" min="2" max="2"/>
-    <col width="61.9" customWidth="1" min="3" max="3"/>
-    <col width="27.2" customWidth="1" min="4" max="4"/>
-    <col width="19.9" customWidth="1" min="5" max="5"/>
-    <col width="15.7" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="68.0"/>
+    <col min="3" max="3" customWidth="true" width="61.9"/>
+    <col min="4" max="4" customWidth="true" width="27.2"/>
+    <col min="5" max="5" customWidth="true" width="19.9"/>
+    <col min="6" max="6" customWidth="true" width="15.7"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1927,8 +1958,9 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1">
+    <row r="4" ht="30.0" customHeight="true">
       <c r="B4" s="2" t="inlineStr">
+        <v>Any rule calls another one by its name with the arguments in parentheses. A name starts with a letter of any script, _ or $ and goes on with letters and digits, as in the rule 면간거리 below. A rule can call itself. When the last parameter is an array, the call can list its elements one by one. A name in back quotes, such as `Rule Name`, may contain any characters.</v>
         <is>
           <t>Any rule calls another one by its name with the arguments in parentheses. A rule can call itself. When the last parameter is an array, the call can list its elements one by one. A name in back quotes, such as `Rule Name`, may contain any characters.</t>
         </is>
@@ -2124,11 +2156,62 @@
         <v>16</v>
       </c>
     </row>
+    <row r="25">
+      <c r="B25" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C31" s="10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>4.0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
EPBDS-9967 Restore K, M, B number multipliers in formulas, exact as in ranges
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
@@ -12,40 +12,9 @@
     <sheet name="Casts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Calls" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Method Double 면간거리(Double 폭, Double 간격)</t>
-  </si>
-  <si>
-    <t>return 폭 + 간격;</t>
-  </si>
-  <si>
-    <t>Test 면간거리 면간거리Test</t>
-  </si>
-  <si>
-    <t>폭</t>
-  </si>
-  <si>
-    <t>Width</t>
-  </si>
-  <si>
-    <t>간격</t>
-  </si>
-  <si>
-    <t>Gap</t>
-  </si>
-  <si>
-    <t>_res_</t>
-  </si>
-  <si>
-    <t>Distance</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -581,27 +550,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:R49"/>
+  <dimension ref="A2:V53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="2.5"/>
-    <col min="2" max="2" customWidth="true" width="24.7"/>
-    <col min="3" max="3" customWidth="true" width="27.9"/>
-    <col min="4" max="4" customWidth="true" width="20.9"/>
-    <col min="5" max="5" customWidth="true" width="21.9"/>
-    <col min="6" max="6" customWidth="true" width="23.0"/>
-    <col min="7" max="7" customWidth="true" width="17.8"/>
-    <col min="8" max="8" customWidth="true" width="23.0"/>
-    <col min="9" max="9" customWidth="true" width="20.9"/>
-    <col min="10" max="10" customWidth="true" width="16.7"/>
-    <col min="11" max="11" customWidth="true" width="16.7"/>
-    <col min="12" max="12" customWidth="true" width="25.1"/>
-    <col min="13" max="13" customWidth="true" width="25.1"/>
-    <col min="14" max="14" customWidth="true" width="27.2"/>
-    <col min="15" max="15" customWidth="true" width="30.4"/>
-    <col min="16" max="16" customWidth="true" width="21.9"/>
-    <col min="17" max="17" customWidth="true" width="21.9"/>
-    <col min="18" max="18" customWidth="true" width="24.1"/>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="24.7" customWidth="1" min="2" max="2"/>
+    <col width="27.9" customWidth="1" min="3" max="3"/>
+    <col width="20.9" customWidth="1" min="4" max="4"/>
+    <col width="21.9" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="17.8" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="20.9" customWidth="1" min="9" max="9"/>
+    <col width="16.7" customWidth="1" min="10" max="10"/>
+    <col width="16.7" customWidth="1" min="11" max="11"/>
+    <col width="25.1" customWidth="1" min="12" max="12"/>
+    <col width="25.1" customWidth="1" min="13" max="13"/>
+    <col width="27.2" customWidth="1" min="14" max="14"/>
+    <col width="30.4" customWidth="1" min="15" max="15"/>
+    <col width="21.9" customWidth="1" min="16" max="16"/>
+    <col width="21.9" customWidth="1" min="17" max="17"/>
+    <col width="24.1" customWidth="1" min="18" max="18"/>
+    <col width="24.1" customWidth="1" min="19" max="19"/>
+    <col width="24.1" customWidth="1" min="20" max="20"/>
+    <col width="24.1" customWidth="1" min="21" max="21"/>
+    <col width="24.1" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -611,17 +584,17 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="43.5" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Formulas accept Java-like literals, written in digits only. A whole number is an Integer, "L" makes it a Long, "0x" starts a hexadecimal number, leading zeros keep a number decimal, a dot or an exponent makes a Double, "f" a Float, and "%" divides by 100 exactly, with any number of decimals.</t>
+          <t>Formulas accept Java-like literals, written in digits only. A whole number is an Integer, "L" makes it a Long, "0x" starts a hexadecimal number, leading zeros keep a number decimal, a dot or an exponent makes a Double, "f" a Float, and "%" divides by 100 exactly, with any number of decimals. "K", "M" and "B" multiply by a thousand, a million and a billion exactly, so 2.5M is the Integer 2500000, 3B is a Long, and 1.0005K is the Double 1000.5.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. "$" starts a reference to a spreadsheet step, so it cannot start a number, and K, M, B are not multipliers. Range cells accept these forms, see the ValuesAndRanges workbook. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
+          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. "$" starts a reference to a spreadsheet step, so it cannot start a number. Range cells accept these forms, see the ValuesAndRanges workbook. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
         </is>
       </c>
     </row>
@@ -849,521 +822,635 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Thousands</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>= 5K</t>
+        </is>
+      </c>
+    </row>
     <row r="28">
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Millions</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>= 2.5M</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Billions</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>= 3B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>ExactThousands</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>= 1.0005K</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Test NumberLiterals NumberLiteralsTest</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="8" t="n"/>
-      <c r="G28" s="8" t="n"/>
-      <c r="H28" s="8" t="n"/>
-      <c r="I28" s="8" t="n"/>
-      <c r="J28" s="8" t="n"/>
-      <c r="K28" s="8" t="n"/>
-      <c r="L28" s="8" t="n"/>
-      <c r="M28" s="8" t="n"/>
-      <c r="N28" s="8" t="n"/>
-      <c r="O28" s="8" t="n"/>
-      <c r="P28" s="8" t="n"/>
-      <c r="Q28" s="8" t="n"/>
-      <c r="R28" s="4" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="9" t="inlineStr">
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8" t="n"/>
+      <c r="K32" s="8" t="n"/>
+      <c r="L32" s="8" t="n"/>
+      <c r="M32" s="8" t="n"/>
+      <c r="N32" s="8" t="n"/>
+      <c r="O32" s="8" t="n"/>
+      <c r="P32" s="8" t="n"/>
+      <c r="Q32" s="8" t="n"/>
+      <c r="R32" s="8" t="n"/>
+      <c r="S32" s="8" t="n"/>
+      <c r="T32" s="8" t="n"/>
+      <c r="U32" s="8" t="n"/>
+      <c r="V32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>_res_.$WholeNumber</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>_res_.$LongNumber</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>_res_.$Hexadecimal</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E33" s="9" t="inlineStr">
         <is>
           <t>_res_.$LeadingZeros</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>_res_.$Fraction</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>_res_.$Exponent</t>
         </is>
       </c>
-      <c r="H29" s="9" t="inlineStr">
+      <c r="H33" s="9" t="inlineStr">
         <is>
           <t>_res_.$LargeExponent</t>
         </is>
       </c>
-      <c r="I29" s="9" t="inlineStr">
+      <c r="I33" s="9" t="inlineStr">
         <is>
           <t>_res_.$FloatNumber</t>
         </is>
       </c>
-      <c r="J29" s="9" t="inlineStr">
+      <c r="J33" s="9" t="inlineStr">
         <is>
           <t>_res_.$Million</t>
         </is>
       </c>
-      <c r="K29" s="9" t="inlineStr">
+      <c r="K33" s="9" t="inlineStr">
         <is>
           <t>_res_.$Percent</t>
         </is>
       </c>
-      <c r="L29" s="9" t="inlineStr">
+      <c r="L33" s="9" t="inlineStr">
         <is>
           <t>_res_.$NegativePercent</t>
         </is>
       </c>
-      <c r="M29" s="9" t="inlineStr">
+      <c r="M33" s="9" t="inlineStr">
         <is>
           <t>_res_.$FractionPercent</t>
         </is>
       </c>
-      <c r="N29" s="9" t="inlineStr">
+      <c r="N33" s="9" t="inlineStr">
         <is>
           <t>_res_.$OneDecimalPercent</t>
         </is>
       </c>
-      <c r="O29" s="9" t="inlineStr">
+      <c r="O33" s="9" t="inlineStr">
         <is>
           <t>_res_.$ThreeDecimalsPercent</t>
         </is>
       </c>
-      <c r="P29" s="9" t="inlineStr">
+      <c r="P33" s="9" t="inlineStr">
         <is>
           <t>_res_.$ExactPercent</t>
         </is>
       </c>
-      <c r="Q29" s="9" t="inlineStr">
+      <c r="Q33" s="9" t="inlineStr">
         <is>
           <t>_res_.$WholePercent</t>
         </is>
       </c>
-      <c r="R29" s="9" t="inlineStr">
+      <c r="R33" s="9" t="inlineStr">
         <is>
           <t>_res_.$CommaSeparates</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="5" t="inlineStr">
+      <c r="S33" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Thousands</t>
+        </is>
+      </c>
+      <c r="T33" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Millions</t>
+        </is>
+      </c>
+      <c r="U33" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Billions</t>
+        </is>
+      </c>
+      <c r="V33" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ExactThousands</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>42L</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>0xFF</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>010</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>1.5e3</t>
         </is>
       </c>
-      <c r="H30" s="5" t="inlineStr">
+      <c r="H34" s="5" t="inlineStr">
         <is>
           <t>1E6</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr">
+      <c r="I34" s="5" t="inlineStr">
         <is>
           <t>2.5f</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr">
+      <c r="J34" s="5" t="inlineStr">
         <is>
           <t>1000000</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="K34" s="5" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="L30" s="5" t="inlineStr">
+      <c r="L34" s="5" t="inlineStr">
         <is>
           <t>-15%</t>
         </is>
       </c>
-      <c r="M30" s="5" t="inlineStr">
+      <c r="M34" s="5" t="inlineStr">
         <is>
           <t>0.25%</t>
         </is>
       </c>
-      <c r="N30" s="5" t="inlineStr">
+      <c r="N34" s="5" t="inlineStr">
         <is>
           <t>0.5%</t>
         </is>
       </c>
-      <c r="O30" s="5" t="inlineStr">
+      <c r="O34" s="5" t="inlineStr">
         <is>
           <t>12.345%</t>
         </is>
       </c>
-      <c r="P30" s="5" t="inlineStr">
+      <c r="P34" s="5" t="inlineStr">
         <is>
           <t>0.07% ==== 0.0007</t>
         </is>
       </c>
-      <c r="Q30" s="5" t="inlineStr">
+      <c r="Q34" s="5" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="R30" s="5" t="inlineStr">
+      <c r="R34" s="5" t="inlineStr">
         <is>
           <t>max(1,000)</t>
         </is>
       </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="10" t="n">
+      <c r="S34" s="5" t="inlineStr">
+        <is>
+          <t>5K</t>
+        </is>
+      </c>
+      <c r="T34" s="5" t="inlineStr">
+        <is>
+          <t>2.5M</t>
+        </is>
+      </c>
+      <c r="U34" s="5" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="V34" s="5" t="inlineStr">
+        <is>
+          <t>1.0005K</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="C31" s="10" t="n">
+      <c r="C35" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="D31" s="10" t="n">
+      <c r="D35" s="10" t="n">
         <v>255</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E35" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="F31" s="10" t="n">
+      <c r="F35" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="G31" s="10" t="n">
+      <c r="G35" s="10" t="n">
         <v>1500</v>
       </c>
-      <c r="H31" s="10" t="n">
+      <c r="H35" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="I31" s="10" t="n">
+      <c r="I35" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="J31" s="10" t="n">
+      <c r="J35" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K31" s="10" t="n">
+      <c r="K35" s="10" t="n">
         <v>0.15</v>
       </c>
-      <c r="L31" s="10" t="n">
+      <c r="L35" s="10" t="n">
         <v>-0.15</v>
       </c>
-      <c r="M31" s="10" t="n">
+      <c r="M35" s="10" t="n">
         <v>0.0025</v>
       </c>
-      <c r="N31" s="10" t="n">
+      <c r="N35" s="10" t="n">
         <v>0.005</v>
       </c>
-      <c r="O31" s="10" t="n">
+      <c r="O35" s="10" t="n">
         <v>0.12345</v>
       </c>
-      <c r="P31" s="10" t="inlineStr">
+      <c r="P35" s="10" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="Q31" s="10" t="n">
+      <c r="Q35" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="R31" s="10" t="n">
+      <c r="R35" s="10" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="2" t="inlineStr">
+      <c r="S35" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="T35" s="10" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="U35" s="10" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="V35" s="10" t="n">
+        <v>1000.5</v>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>A text is in double quotes and a character in single quotes. A backslash escapes special characters: \n a new line, \t a tab, \" a quote, \\ a backslash, \u00e9 a Unicode character. true, false and null are the Boolean and empty values.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="3" t="inlineStr">
+    <row r="38"/>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult TextLiterals()</t>
         </is>
       </c>
-      <c r="C35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="5" t="inlineStr">
+      <c r="C39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>= "Hello"</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>Character</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>= 'A'</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>Quoted</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>= "Say \"Hi\""</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>QuotedLength</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>= length($Quoted)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>NewLineLength</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>= length("Line\nBreak")</t>
+          <t>= "Hello"</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Unicode</t>
+          <t>Character</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>= "Caf\u00e9"</t>
+          <t>= 'A'</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Quoted</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>= true</t>
+          <t>= "Say \"Hi\""</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="6" t="inlineStr">
         <is>
+          <t>QuotedLength</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>= length($Quoted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>NewLineLength</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>= length("Line\nBreak")</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>Unicode</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>= "Caf\u00e9"</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>= true</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="6" t="inlineStr">
+        <is>
           <t>Nothing</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>= null</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Test TextLiterals TextLiteralsTest</t>
         </is>
       </c>
-      <c r="C46" s="8" t="n"/>
-      <c r="D46" s="8" t="n"/>
-      <c r="E46" s="8" t="n"/>
-      <c r="F46" s="8" t="n"/>
-      <c r="G46" s="8" t="n"/>
-      <c r="H46" s="8" t="n"/>
-      <c r="I46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="9" t="inlineStr">
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Text</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Character</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Quoted</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr">
         <is>
           <t>_res_.$QuotedLength</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>_res_.$NewLineLength</t>
         </is>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="G51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Unicode</t>
         </is>
       </c>
-      <c r="H47" s="9" t="inlineStr">
+      <c r="H51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Yes</t>
         </is>
       </c>
-      <c r="I47" s="9" t="inlineStr">
+      <c r="I51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Nothing</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="5" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>Character</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>Quoted</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>Quoted Length</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr">
+      <c r="F52" s="5" t="inlineStr">
         <is>
           <t>New Line Length</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G52" s="5" t="inlineStr">
         <is>
           <t>Unicode</t>
         </is>
       </c>
-      <c r="H48" s="5" t="inlineStr">
+      <c r="H52" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I48" s="5" t="inlineStr">
+      <c r="I52" s="5" t="inlineStr">
         <is>
           <t>Nothing</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="10" t="inlineStr">
+    <row r="53">
+      <c r="B53" s="10" t="inlineStr">
         <is>
           <t>Hello</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D49" s="10" t="inlineStr">
+      <c r="D53" s="10" t="inlineStr">
         <is>
           <t>Say "Hi"</t>
         </is>
       </c>
-      <c r="E49" s="10" t="n">
+      <c r="E53" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="F49" s="10" t="n">
+      <c r="F53" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G49" s="10" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="H49" s="10" t="inlineStr">
+      <c r="H53" s="10" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="I49" s="10" t="n"/>
-    </row>
+      <c r="I53" s="10" t="n"/>
+    </row>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B50:I50"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B28:R28"/>
-    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B32:V32"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B35:C35"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1377,15 +1464,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F16"/>
+  <dimension ref="B2:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="2.5"/>
-    <col min="2" max="2" customWidth="true" width="16.8"/>
-    <col min="3" max="3" customWidth="true" width="72.2"/>
-    <col min="4" max="4" customWidth="true" width="14.6"/>
-    <col min="5" max="5" customWidth="true" width="21.9"/>
-    <col min="6" max="6" customWidth="true" width="21.9"/>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="16.8" customWidth="1" min="2" max="2"/>
+    <col width="72.2" customWidth="1" min="3" max="3"/>
+    <col width="14.6" customWidth="1" min="4" max="4"/>
+    <col width="21.9" customWidth="1" min="5" max="5"/>
+    <col width="21.9" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1577,15 +1664,15 @@
   <dimension ref="B2:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="2.5"/>
-    <col min="2" max="2" customWidth="true" width="42.7"/>
-    <col min="3" max="3" customWidth="true" width="50.3"/>
-    <col min="4" max="4" customWidth="true" width="15.7"/>
-    <col min="5" max="5" customWidth="true" width="21.9"/>
-    <col min="6" max="6" customWidth="true" width="25.1"/>
-    <col min="7" max="7" customWidth="true" width="14.6"/>
-    <col min="8" max="8" customWidth="true" width="15.7"/>
-    <col min="9" max="9" customWidth="true" width="19.9"/>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="42.7" customWidth="1" min="2" max="2"/>
+    <col width="50.3" customWidth="1" min="3" max="3"/>
+    <col width="15.7" customWidth="1" min="4" max="4"/>
+    <col width="21.9" customWidth="1" min="5" max="5"/>
+    <col width="25.1" customWidth="1" min="6" max="6"/>
+    <col width="14.6" customWidth="1" min="7" max="7"/>
+    <col width="15.7" customWidth="1" min="8" max="8"/>
+    <col width="19.9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1940,15 +2027,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:F31"/>
+  <dimension ref="B2:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="2.5"/>
-    <col min="2" max="2" customWidth="true" width="68.0"/>
-    <col min="3" max="3" customWidth="true" width="61.9"/>
-    <col min="4" max="4" customWidth="true" width="27.2"/>
-    <col min="5" max="5" customWidth="true" width="19.9"/>
-    <col min="6" max="6" customWidth="true" width="15.7"/>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="68" customWidth="1" min="2" max="2"/>
+    <col width="61.9" customWidth="1" min="3" max="3"/>
+    <col width="27.2" customWidth="1" min="4" max="4"/>
+    <col width="19.9" customWidth="1" min="5" max="5"/>
+    <col width="15.7" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1958,9 +2045,8 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="30.0" customHeight="true">
+    <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
-        <v>Any rule calls another one by its name with the arguments in parentheses. A name starts with a letter of any script, _ or $ and goes on with letters and digits, as in the rule 면간거리 below. A rule can call itself. When the last parameter is an array, the call can list its elements one by one. A name in back quotes, such as `Rule Name`, may contain any characters.</v>
         <is>
           <t>Any rule calls another one by its name with the arguments in parentheses. A rule can call itself. When the last parameter is an array, the call can list its elements one by one. A name in back quotes, such as `Rule Name`, may contain any characters.</t>
         </is>
@@ -2157,42 +2243,60 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="3" t="s">
-        <v>0</v>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Method Double 면간거리(Double 폭, Double 간격)</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="6" t="s">
-        <v>1</v>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>return 폭 + 간격;</t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Test 면간거리 면간거리Test</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="4" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="9" t="s">
-        <v>7</v>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>폭</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>간격</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>8</v>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Width</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -2203,14 +2307,14 @@
         <v>1.5</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>4.0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
EPBDS-9967 Remove the $ currency sign from range numbers, so no number takes it
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
@@ -550,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:V53"/>
+  <dimension ref="B2:V53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -594,7 +594,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. "$" starts a reference to a spreadsheet step, so it cannot start a number. Range cells accept these forms, see the ValuesAndRanges workbook. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
+          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. Range cells group thousands, see the ValuesAndRanges workbook. "$" starts a reference to a spreadsheet step and is never a part of a number. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -1179,7 +1178,6 @@
         <v>1000.5</v>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -1187,7 +1185,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -1304,7 +1301,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="B50" s="3" t="inlineStr">
         <is>
@@ -1437,12 +1433,6 @@
       </c>
       <c r="I53" s="10" t="n"/>
     </row>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B39:C39"/>

</xml_diff>

<commit_message>
EPBDS-9967 Read commas grouping thousands by three digits in number cells and formulas
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Expressions.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Statements" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Casts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Calls" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Pitfalls" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -550,7 +551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:V53"/>
+  <dimension ref="B2:X55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -575,6 +576,8 @@
     <col width="24.1" customWidth="1" min="20" max="20"/>
     <col width="24.1" customWidth="1" min="21" max="21"/>
     <col width="24.1" customWidth="1" min="22" max="22"/>
+    <col width="24.1" customWidth="1" min="23" max="23"/>
+    <col width="24.1" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -587,14 +590,14 @@
     <row r="4" ht="43.5" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Formulas accept Java-like literals, written in digits only. A whole number is an Integer, "L" makes it a Long, "0x" starts a hexadecimal number, leading zeros keep a number decimal, a dot or an exponent makes a Double, "f" a Float, and "%" divides by 100 exactly, with any number of decimals. "K", "M" and "B" multiply by a thousand, a million and a billion exactly, so 2.5M is the Integer 2500000, 3B is a Long, and 1.0005K is the Double 1000.5.</t>
+          <t>Formulas accept Java-like literals. A whole number is an Integer, "L" makes it a Long, "0x" starts a hexadecimal number, leading zeros keep a number decimal, a dot or an exponent makes a Double, "f" a Float, and "%" divides by 100 exactly, with any number of decimals. "K", "M" and "B" multiply by a thousand, a million and a billion exactly, so 2.5M is the Integer 2500000, 3B is a Long, and 1.0005K is the Double 1000.5. Commas group the thousands of a number that starts with 1 to 9, three digits per group: 12,345,678 and 1,000.50.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>A comma always separates values, so it cannot group thousands: max(1,000) compares 1 with 0. Range cells group thousands, see the ValuesAndRanges workbook. "$" starts a reference to a spreadsheet step and is never a part of a number. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
+          <t>Any other comma separates values: max(12,34), max(1, 500) and max(0,500) compare two numbers, while 12,34.00 and 1,00,000 are not numbers. The Pitfalls sheet shows more commas in arrays and arguments. "$" starts a reference to a spreadsheet step and is never a part of a number. There are no octal numbers: 010 is 10, and Date(2021, 04, 08) is Date(2021, 4, 8).</t>
         </is>
       </c>
     </row>
@@ -818,7 +821,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>= max(1,000)</t>
+          <t>= max(12,34)</t>
         </is>
       </c>
     </row>
@@ -870,576 +873,628 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>GroupedWhole</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>= 12,345,678</t>
+        </is>
+      </c>
+    </row>
     <row r="32">
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>GroupedFraction</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>= 1,000.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Test NumberLiterals NumberLiteralsTest</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="8" t="n"/>
-      <c r="G32" s="8" t="n"/>
-      <c r="H32" s="8" t="n"/>
-      <c r="I32" s="8" t="n"/>
-      <c r="J32" s="8" t="n"/>
-      <c r="K32" s="8" t="n"/>
-      <c r="L32" s="8" t="n"/>
-      <c r="M32" s="8" t="n"/>
-      <c r="N32" s="8" t="n"/>
-      <c r="O32" s="8" t="n"/>
-      <c r="P32" s="8" t="n"/>
-      <c r="Q32" s="8" t="n"/>
-      <c r="R32" s="8" t="n"/>
-      <c r="S32" s="8" t="n"/>
-      <c r="T32" s="8" t="n"/>
-      <c r="U32" s="8" t="n"/>
-      <c r="V32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="9" t="inlineStr">
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
+      <c r="K34" s="8" t="n"/>
+      <c r="L34" s="8" t="n"/>
+      <c r="M34" s="8" t="n"/>
+      <c r="N34" s="8" t="n"/>
+      <c r="O34" s="8" t="n"/>
+      <c r="P34" s="8" t="n"/>
+      <c r="Q34" s="8" t="n"/>
+      <c r="R34" s="8" t="n"/>
+      <c r="S34" s="8" t="n"/>
+      <c r="T34" s="8" t="n"/>
+      <c r="U34" s="8" t="n"/>
+      <c r="V34" s="8" t="n"/>
+      <c r="W34" s="8" t="n"/>
+      <c r="X34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>_res_.$WholeNumber</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>_res_.$LongNumber</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Hexadecimal</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>_res_.$LeadingZeros</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Fraction</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Exponent</t>
         </is>
       </c>
-      <c r="H33" s="9" t="inlineStr">
+      <c r="H35" s="9" t="inlineStr">
         <is>
           <t>_res_.$LargeExponent</t>
         </is>
       </c>
-      <c r="I33" s="9" t="inlineStr">
+      <c r="I35" s="9" t="inlineStr">
         <is>
           <t>_res_.$FloatNumber</t>
         </is>
       </c>
-      <c r="J33" s="9" t="inlineStr">
+      <c r="J35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Million</t>
         </is>
       </c>
-      <c r="K33" s="9" t="inlineStr">
+      <c r="K35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Percent</t>
         </is>
       </c>
-      <c r="L33" s="9" t="inlineStr">
+      <c r="L35" s="9" t="inlineStr">
         <is>
           <t>_res_.$NegativePercent</t>
         </is>
       </c>
-      <c r="M33" s="9" t="inlineStr">
+      <c r="M35" s="9" t="inlineStr">
         <is>
           <t>_res_.$FractionPercent</t>
         </is>
       </c>
-      <c r="N33" s="9" t="inlineStr">
+      <c r="N35" s="9" t="inlineStr">
         <is>
           <t>_res_.$OneDecimalPercent</t>
         </is>
       </c>
-      <c r="O33" s="9" t="inlineStr">
+      <c r="O35" s="9" t="inlineStr">
         <is>
           <t>_res_.$ThreeDecimalsPercent</t>
         </is>
       </c>
-      <c r="P33" s="9" t="inlineStr">
+      <c r="P35" s="9" t="inlineStr">
         <is>
           <t>_res_.$ExactPercent</t>
         </is>
       </c>
-      <c r="Q33" s="9" t="inlineStr">
+      <c r="Q35" s="9" t="inlineStr">
         <is>
           <t>_res_.$WholePercent</t>
         </is>
       </c>
-      <c r="R33" s="9" t="inlineStr">
+      <c r="R35" s="9" t="inlineStr">
         <is>
           <t>_res_.$CommaSeparates</t>
         </is>
       </c>
-      <c r="S33" s="9" t="inlineStr">
+      <c r="S35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Thousands</t>
         </is>
       </c>
-      <c r="T33" s="9" t="inlineStr">
+      <c r="T35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Millions</t>
         </is>
       </c>
-      <c r="U33" s="9" t="inlineStr">
+      <c r="U35" s="9" t="inlineStr">
         <is>
           <t>_res_.$Billions</t>
         </is>
       </c>
-      <c r="V33" s="9" t="inlineStr">
+      <c r="V35" s="9" t="inlineStr">
         <is>
           <t>_res_.$ExactThousands</t>
         </is>
       </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="5" t="inlineStr">
+      <c r="W35" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$GroupedWhole</t>
+        </is>
+      </c>
+      <c r="X35" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$GroupedFraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>42L</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>0xFF</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>010</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>1.5e3</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>1E6</t>
         </is>
       </c>
-      <c r="I34" s="5" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>2.5f</t>
         </is>
       </c>
-      <c r="J34" s="5" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>1000000</t>
         </is>
       </c>
-      <c r="K34" s="5" t="inlineStr">
+      <c r="K36" s="5" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr">
+      <c r="L36" s="5" t="inlineStr">
         <is>
           <t>-15%</t>
         </is>
       </c>
-      <c r="M34" s="5" t="inlineStr">
+      <c r="M36" s="5" t="inlineStr">
         <is>
           <t>0.25%</t>
         </is>
       </c>
-      <c r="N34" s="5" t="inlineStr">
+      <c r="N36" s="5" t="inlineStr">
         <is>
           <t>0.5%</t>
         </is>
       </c>
-      <c r="O34" s="5" t="inlineStr">
+      <c r="O36" s="5" t="inlineStr">
         <is>
           <t>12.345%</t>
         </is>
       </c>
-      <c r="P34" s="5" t="inlineStr">
+      <c r="P36" s="5" t="inlineStr">
         <is>
           <t>0.07% ==== 0.0007</t>
         </is>
       </c>
-      <c r="Q34" s="5" t="inlineStr">
+      <c r="Q36" s="5" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="R34" s="5" t="inlineStr">
-        <is>
-          <t>max(1,000)</t>
-        </is>
-      </c>
-      <c r="S34" s="5" t="inlineStr">
+      <c r="R36" s="5" t="inlineStr">
+        <is>
+          <t>max(12,34)</t>
+        </is>
+      </c>
+      <c r="S36" s="5" t="inlineStr">
         <is>
           <t>5K</t>
         </is>
       </c>
-      <c r="T34" s="5" t="inlineStr">
+      <c r="T36" s="5" t="inlineStr">
         <is>
           <t>2.5M</t>
         </is>
       </c>
-      <c r="U34" s="5" t="inlineStr">
+      <c r="U36" s="5" t="inlineStr">
         <is>
           <t>3B</t>
         </is>
       </c>
-      <c r="V34" s="5" t="inlineStr">
+      <c r="V36" s="5" t="inlineStr">
         <is>
           <t>1.0005K</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="10" t="n">
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>12,345,678</t>
+        </is>
+      </c>
+      <c r="X36" s="5" t="inlineStr">
+        <is>
+          <t>1,000.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="C35" s="10" t="n">
+      <c r="C37" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="D35" s="10" t="n">
+      <c r="D37" s="10" t="n">
         <v>255</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E37" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="F35" s="10" t="n">
+      <c r="F37" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="G35" s="10" t="n">
+      <c r="G37" s="10" t="n">
         <v>1500</v>
       </c>
-      <c r="H35" s="10" t="n">
+      <c r="H37" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="I35" s="10" t="n">
+      <c r="I37" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="J35" s="10" t="n">
+      <c r="J37" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="K35" s="10" t="n">
+      <c r="K37" s="10" t="n">
         <v>0.15</v>
       </c>
-      <c r="L35" s="10" t="n">
+      <c r="L37" s="10" t="n">
         <v>-0.15</v>
       </c>
-      <c r="M35" s="10" t="n">
+      <c r="M37" s="10" t="n">
         <v>0.0025</v>
       </c>
-      <c r="N35" s="10" t="n">
+      <c r="N37" s="10" t="n">
         <v>0.005</v>
       </c>
-      <c r="O35" s="10" t="n">
+      <c r="O37" s="10" t="n">
         <v>0.12345</v>
       </c>
-      <c r="P35" s="10" t="inlineStr">
+      <c r="P37" s="10" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="Q35" s="10" t="n">
+      <c r="Q37" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="R35" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="S35" s="10" t="n">
+      <c r="R37" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="S37" s="10" t="n">
         <v>5000</v>
       </c>
-      <c r="T35" s="10" t="n">
+      <c r="T37" s="10" t="n">
         <v>2500000</v>
       </c>
-      <c r="U35" s="10" t="n">
+      <c r="U37" s="10" t="n">
         <v>3000000000</v>
       </c>
-      <c r="V35" s="10" t="n">
+      <c r="V37" s="10" t="n">
         <v>1000.5</v>
       </c>
-    </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="B37" s="2" t="inlineStr">
+      <c r="W37" s="10" t="n">
+        <v>12345678</v>
+      </c>
+      <c r="X37" s="10" t="n">
+        <v>1000.5</v>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>A text is in double quotes and a character in single quotes. A backslash escapes special characters: \n a new line, \t a tab, \" a quote, \\ a backslash, \u00e9 a Unicode character. true, false and null are the Boolean and empty values.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="3" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult TextLiterals()</t>
         </is>
       </c>
-      <c r="C39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="5" t="inlineStr">
+      <c r="C41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>= "Hello"</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>Character</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>= 'A'</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Quoted</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>= "Say \"Hi\""</t>
+          <t>= "Hello"</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>QuotedLength</t>
+          <t>Character</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>= length($Quoted)</t>
+          <t>= 'A'</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>NewLineLength</t>
+          <t>Quoted</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>= length("Line\nBreak")</t>
+          <t>= "Say \"Hi\""</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Unicode</t>
+          <t>QuotedLength</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>= "Caf\u00e9"</t>
+          <t>= length($Quoted)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NewLineLength</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>= true</t>
+          <t>= length("Line\nBreak")</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="6" t="inlineStr">
         <is>
+          <t>Unicode</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>= "Caf\u00e9"</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>= true</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="6" t="inlineStr">
+        <is>
           <t>Nothing</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>= null</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="3" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Test TextLiterals TextLiteralsTest</t>
         </is>
       </c>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="8" t="n"/>
-      <c r="F50" s="8" t="n"/>
-      <c r="G50" s="8" t="n"/>
-      <c r="H50" s="8" t="n"/>
-      <c r="I50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="9" t="inlineStr">
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="8" t="n"/>
+      <c r="I52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="9" t="inlineStr">
         <is>
           <t>_res_.$Text</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C53" s="9" t="inlineStr">
         <is>
           <t>_res_.$Character</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D53" s="9" t="inlineStr">
         <is>
           <t>_res_.$Quoted</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E53" s="9" t="inlineStr">
         <is>
           <t>_res_.$QuotedLength</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="F53" s="9" t="inlineStr">
         <is>
           <t>_res_.$NewLineLength</t>
         </is>
       </c>
-      <c r="G51" s="9" t="inlineStr">
+      <c r="G53" s="9" t="inlineStr">
         <is>
           <t>_res_.$Unicode</t>
         </is>
       </c>
-      <c r="H51" s="9" t="inlineStr">
+      <c r="H53" s="9" t="inlineStr">
         <is>
           <t>_res_.$Yes</t>
         </is>
       </c>
-      <c r="I51" s="9" t="inlineStr">
+      <c r="I53" s="9" t="inlineStr">
         <is>
           <t>_res_.$Nothing</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="5" t="inlineStr">
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Character</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Quoted</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>Quoted Length</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>New Line Length</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="G54" s="5" t="inlineStr">
         <is>
           <t>Unicode</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="H54" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I52" s="5" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr">
         <is>
           <t>Nothing</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="10" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>Hello</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="D55" s="10" t="inlineStr">
         <is>
           <t>Say "Hi"</t>
         </is>
       </c>
-      <c r="E53" s="10" t="n">
+      <c r="E55" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="F53" s="10" t="n">
+      <c r="F55" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="G53" s="10" t="inlineStr">
+      <c r="G55" s="10" t="inlineStr">
         <is>
           <t>Café</t>
         </is>
       </c>
-      <c r="H53" s="10" t="inlineStr">
+      <c r="H55" s="10" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="I53" s="10" t="n"/>
+      <c r="I55" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B34:X34"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B32:V32"/>
+    <mergeCell ref="B41:C41"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
@@ -2310,4 +2365,381 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:L23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="24.7" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="20.9" customWidth="1" min="4" max="4"/>
+    <col width="21.9" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="17.8" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="20.9" customWidth="1" min="9" max="9"/>
+    <col width="16.7" customWidth="1" min="10" max="10"/>
+    <col width="16.7" customWidth="1" min="11" max="11"/>
+    <col width="25.1" customWidth="1" min="12" max="12"/>
+    <col width="25.1" customWidth="1" min="13" max="13"/>
+    <col width="27.2" customWidth="1" min="14" max="14"/>
+    <col width="30.4" customWidth="1" min="15" max="15"/>
+    <col width="21.9" customWidth="1" min="16" max="16"/>
+    <col width="21.9" customWidth="1" min="17" max="17"/>
+    <col width="24.1" customWidth="1" min="18" max="18"/>
+    <col width="24.1" customWidth="1" min="19" max="19"/>
+    <col width="24.1" customWidth="1" min="20" max="20"/>
+    <col width="24.1" customWidth="1" min="21" max="21"/>
+    <col width="24.1" customWidth="1" min="22" max="22"/>
+    <col width="24.1" customWidth="1" min="23" max="23"/>
+    <col width="24.1" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Pitfalls of ambiguous syntax</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>A comma between digits in an array or in the arguments of a function groups thousands when the number starts with 1 to 9 and every next group has three digits, so {10,500,600} holds one number. Any other comma separates values. Write a space after a comma that separates values: {10, 500, 600} holds three numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult CommaInLists()</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>OneGroupedNumber</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>= Integer[] a = new Integer[] {1,000}; a.length</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>SpaceSeparates</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>= Integer[] a = new Integer[] {1, 000}; a.length</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>GroupedElement</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>= new Integer[] {10,500,600}[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>ThreeElements</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>= Integer[] a = new Integer[] {10, 500, 600}; a.length</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>ShortLastGroup</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>= Integer[] a = new Integer[] {1,000,2}; a.length</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>LeadingZero</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>= Integer[] a = new Integer[] {0,500}; a.length</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>ShortGroup</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>= Integer[] a = new Integer[] {12,34}; a.length</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>TwoGroupedArguments</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>= max(1,000, 2,500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>FourArguments</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>= max(1, 000, 2, 500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>GroupedFractions</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>= max(1,000.5, 999.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>RoundGrouped</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>= round(1,234.567, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Test CommaInLists CommaInListsTest</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
+      <c r="L20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$OneGroupedNumber</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$SpaceSeparates</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$GroupedElement</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ThreeElements</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ShortLastGroup</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$LeadingZero</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ShortGroup</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$TwoGroupedArguments</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FourArguments</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$GroupedFractions</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$RoundGrouped</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Integer[] a = new Integer[] {1,000}; a.length</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Integer[] a = new Integer[] {1, 000}; a.length</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>new Integer[] {10,500,600}[0]</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Integer[] a = new Integer[] {10, 500, 600}; a.length</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Integer[] a = new Integer[] {1,000,2}; a.length</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Integer[] a = new Integer[] {0,500}; a.length</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Integer[] a = new Integer[] {12,34}; a.length</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>max(1,000, 2,500)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>max(1, 000, 2, 500)</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>max(1,000.5, 999.5)</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>round(1,234.567, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>10500600</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" s="10" t="n">
+        <v>2500</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>1000.5</v>
+      </c>
+      <c r="L23" s="10" t="n">
+        <v>1234.57</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B20:L20"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B4:I4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>